<commit_message>
cambiati archon per test
</commit_message>
<xml_diff>
--- a/vtesitaly/assets/archon/archon.xlsx
+++ b/vtesitaly/assets/archon/archon.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
   <si>
     <t>#</t>
   </si>
@@ -25,6 +25,51 @@
   </si>
   <si>
     <t>Table#</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>Francesco</t>
+  </si>
+  <si>
+    <t>Rampionesi</t>
+  </si>
+  <si>
+    <t>2</t>
+  </si>
+  <si>
+    <t>Simone</t>
+  </si>
+  <si>
+    <t>Parmeggiani</t>
+  </si>
+  <si>
+    <t>3</t>
+  </si>
+  <si>
+    <t>Lovre</t>
+  </si>
+  <si>
+    <t xml:space="preserve">De Grisogono</t>
+  </si>
+  <si>
+    <t>4</t>
+  </si>
+  <si>
+    <t>Miro</t>
+  </si>
+  <si>
+    <t>Albertazzi</t>
+  </si>
+  <si>
+    <t>5</t>
+  </si>
+  <si>
+    <t>Stefano</t>
+  </si>
+  <si>
+    <t>Chiodi</t>
   </si>
 </sst>
 </file>
@@ -570,7 +615,10 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="4" style="1" width="9.140625"/>
+    <col min="1" max="1" style="1" width="9.140625"/>
+    <col customWidth="1" min="2" max="2" style="1" width="11.421875"/>
+    <col customWidth="1" min="3" max="3" style="1" width="12.7109375"/>
+    <col min="4" max="4" style="1" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" ht="14.25">
@@ -588,34 +636,74 @@
       </c>
     </row>
     <row r="2" ht="14.25">
-      <c r="A2" s="1"/>
-      <c r="B2" s="1"/>
-      <c r="C2" s="1"/>
-      <c r="D2" s="1"/>
+      <c r="A2" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="3" ht="14.25">
-      <c r="A3" s="1"/>
-      <c r="B3" s="1"/>
-      <c r="C3" s="1"/>
-      <c r="D3" s="1"/>
+      <c r="A3" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="4" ht="14.25">
-      <c r="A4" s="1"/>
-      <c r="B4" s="1"/>
-      <c r="C4" s="1"/>
-      <c r="D4" s="1"/>
+      <c r="A4" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="5" ht="14.25">
-      <c r="A5" s="1"/>
-      <c r="B5" s="1"/>
-      <c r="C5" s="1"/>
-      <c r="D5" s="1"/>
+      <c r="A5" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="6" ht="14.25">
-      <c r="A6" s="1"/>
-      <c r="B6" s="1"/>
-      <c r="C6" s="1"/>
-      <c r="D6" s="1"/>
+      <c r="A6" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="7" ht="14.25">
       <c r="A7" s="1"/>

</xml_diff>